<commit_message>
Added Interval sweep algorithms
</commit_message>
<xml_diff>
--- a/DSA/Sorting/dsa_cheatsheet.xlsx
+++ b/DSA/Sorting/dsa_cheatsheet.xlsx
@@ -8,19 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/balaji.gurusala/Documents/Code/coding/DSA/Sorting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334426BD-E91D-2648-A1BC-93D7190B18F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE417D1-D94F-EB43-B21C-E9B0F367709A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Algorithms" sheetId="1" r:id="rId1"/>
+    <sheet name="Pattern Dev." sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="204">
   <si>
     <t>Algorithm / Concept</t>
   </si>
@@ -605,13 +619,407 @@
   </si>
   <si>
     <t>O(1) best / O(n) average / O(n) worst (Amortized linear time due to O(1) hash map lookups)</t>
+  </si>
+  <si>
+    <t>Heap Sort</t>
+  </si>
+  <si>
+    <t>Selection / Tree-Based Priority Queue</t>
+  </si>
+  <si>
+    <t>The Pyramid Bracket: Shape the array into a strict corporate pyramid where parents are always larger than children (Max-Heap). Repeatedly pluck the top boss from the pyramid, swap them to the far right, and force the replacement to sift down to its correct level.</t>
+  </si>
+  <si>
+    <t>1. Build Heap: Loop parent from len(A)//2 - 1 down to 0, calling heapify(A, parent, len(A)). 2. Sort: Loop i from len(A)-1 down to 1. Swap A[0] with A[i], then call heapify(A, 0, i) to sift the new root down within the reduced active heap size.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst (Build phase takes O(n), extraction phase takes O(n log n))</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary (In-place array manipulation.</t>
+  </si>
+  <si>
+    <t>Binary Search (Recursive)</t>
+  </si>
+  <si>
+    <t>Decrease &amp; Conquer (Divide by 2) / Logarithmic Search</t>
+  </si>
+  <si>
+    <t>The Phone Book Flip: Open a sorted book directly to the middle. If the name is further down, throw away the left half entirely and repeat the split on the remaining right half.</t>
+  </si>
+  <si>
+    <t>Base case: if start &gt; end return -1. mid = start + (end - start) // 2. If target &gt; A[mid], return recurse(mid + 1, end). If target &lt; A[mid], return recurse(start, mid - 1). Else, return mid.</t>
+  </si>
+  <si>
+    <t>O(1) best / O(log n) average / O(log n) worst</t>
+  </si>
+  <si>
+    <t>Binary Search (Loop Method)</t>
+  </si>
+  <si>
+    <t>The Book Chopper: Stand over a sorted phone book. Slam your hand directly onto the middle page. If your target is smaller, slice off and discard the entire right half of the book. Repeat on the remaining pages until you land on the name or the pages run out.</t>
+  </si>
+  <si>
+    <t>Initialize start = 0, end = len(A) - 1. Run while start &lt;= end. Calculate mid = start + (end - start) // 2 inside the loop. If target == A[mid], return mid. If target &gt; A[mid], shift start = mid + 1. Else, shift end = mid - 1. Return -1 if loop exits naturally.</t>
+  </si>
+  <si>
+    <t>O(log n) auxiliary space (due to the recursive call stack depth)</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary space (Fixed pointers; completely avoids the O(log n) call stack overhead of the recursive variant)</t>
+  </si>
+  <si>
+    <t>🗂️ Universal Pattern Development Meta-Framework</t>
+  </si>
+  <si>
+    <t>Algorithmic Paradigm</t>
+  </si>
+  <si>
+    <t>Architectural Strategy &amp; Core Mechanics</t>
+  </si>
+  <si>
+    <t>Time Complexity (General)</t>
+  </si>
+  <si>
+    <t>Space Complexity (Auxiliary)</t>
+  </si>
+  <si>
+    <t>Retrospective Pro/Con &amp; Whiteboard Invariant</t>
+  </si>
+  <si>
+    <t>1. Brute Force</t>
+  </si>
+  <si>
+    <t>• Mechanics: The baseline implementation. Uses nested loops or naive exhaustive search to check all possibilities.
+• Whiteboard Role: Validates problem understanding; serves as the rock-solid stepping stone for optimization.</t>
+  </si>
+  <si>
+    <t>O(1)</t>
+  </si>
+  <si>
+    <t>Pro: Extremely simple, zero memory overhead.Con: Highly expensive, unacceptable for production-scale data.</t>
+  </si>
+  <si>
+    <t>2. Decrease &amp; Conquer</t>
+  </si>
+  <si>
+    <t>• Mechanics: Reduces the problem size step-by-step by processing one element at a time (often working at the end/boundaries).• Recurrence: \(T(n) = T(n-1) + O(n)\) (e.g., Insertion Sort).</t>
+  </si>
+  <si>
+    <t>O(nlogn)</t>
+  </si>
+  <si>
+    <t>O(n) - Merge and O(logn) for quick sort</t>
+  </si>
+  <si>
+    <t>Pro: Breaks down large datasets efficiently.Con: Stack depth overhead; combining sub-problems often requires extra memory.</t>
+  </si>
+  <si>
+    <t>O(n^2)</t>
+  </si>
+  <si>
+    <t>O(n^2)  to O(2^n)</t>
+  </si>
+  <si>
+    <t>O(1) - Iterative O(n) - Recursive</t>
+  </si>
+  <si>
+    <t>Pro: Intuitive boundary transitions.Con: Still bound to quadratic limits if every step requires a linear scan</t>
+  </si>
+  <si>
+    <t>3. Divide &amp; Conquer</t>
+  </si>
+  <si>
+    <t>• Mechanics: Splitting the problem into independent sub-problems, solving them, and combining results.• Work Profiles: Work upfront to partition (QuickSort) OR work at the end to combine/merge (MergeSort).</t>
+  </si>
+  <si>
+    <t>4. Transform &amp; Conquer(Data Structure Shift)</t>
+  </si>
+  <si>
+    <t>• Mechanics: Converts the raw input into an optimized data structure to change the rules of retrieval.
+• Heaps vs. BSTs: A Max/Min Heap builds in (O(n)), sorts in O(nlogn)  but searching takes (O(n)) using two pointer pass etc.. A Balanced BST builds in (O(n log n)) but allows searching in (O(log n)).</t>
+  </si>
+  <si>
+    <t>Pro: Excellent for top-K, priority tracking, or continuous dynamic data.
+Con: High pointer allocation overhead or restricted internal search access.</t>
+  </si>
+  <si>
+    <t>O(n)</t>
+  </si>
+  <si>
+    <t>5. Transform &amp; Conquer(Pre-Sorting Step)</t>
+  </si>
+  <si>
+    <t>• Mechanics: Sorts the array as an explicit pre-processing step ((O(n log n))) to unlock highly optimized downstream passes.
+• Downstream Patterns: Unlocks Two-Pointer Pincer Scans ((O(n))) or Binary Search sweeps ((O(log n))).</t>
+  </si>
+  <si>
+    <t>Pro: Zero auxiliary space required (if sorted in-place). Permanent whiteboard fallback.
+Con: Hard-capped by the (O(n log n)) sorting bottleneck.</t>
+  </si>
+  <si>
+    <t>6. Space-Time Trade-off(Hash Table Lookup)</t>
+  </si>
+  <si>
+    <t>• Mechanics: Allocates memory dynamically to store state or frequencies, dropping lookup times from linear to constant.
+• Optimization: Interleaves the Build + Search processes into a Single Pass to find complements on the fly.</t>
+  </si>
+  <si>
+    <t>Pro: Maximum possible time efficiency (linear speed)
+.Con: High auxiliary space cost. Vulnerable to hash collision edge cases.</t>
+  </si>
+  <si>
+    <t>Algorithms to try</t>
+  </si>
+  <si>
+    <t>* Bubble Sort, Selection</t>
+  </si>
+  <si>
+    <t>* Insertion sort</t>
+  </si>
+  <si>
+    <t>Quick Sort, Merge Sort</t>
+  </si>
+  <si>
+    <t>Min Heap, Max Heap, BST</t>
+  </si>
+  <si>
+    <t>Pre Sorting + Binary Search or Two Pointer pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HashMap </t>
+  </si>
+  <si>
+    <t>Kth Largest via Full Sorting (Brute Force)</t>
+  </si>
+  <si>
+    <t>Brute Force / Exhaustive Transformation</t>
+  </si>
+  <si>
+    <t>The Complete Overhaul: Sort the entire unsorted crowd from largest to smallest first, then walk directly to the Kth seat to read the answer.</t>
+  </si>
+  <si>
+    <t>Sort the entire array A using a standard O(n log n) sorting library call. Return the element directly using fixed index lookup: A[len(A) - k] for ascending sort or A[k - 1] for descending sort.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst (Capped by the initial sorting routine)</t>
+  </si>
+  <si>
+    <t>O(1) to O(n) auxiliary (Dependent entirely on the internal space requirement of the language's sorting engine)</t>
+  </si>
+  <si>
+    <t>Kth Largest via Partial Selection/Bubble Scan</t>
+  </si>
+  <si>
+    <t>Decrease &amp; Conquer (Reduce search space on boundaries)</t>
+  </si>
+  <si>
+    <t>The Sequential Extractor: Run a forward scan to find the absolute largest item and push it to the far right. Repeat this boundary scan exactly K times to lock in the top K positions, ignoring the rest.</t>
+  </si>
+  <si>
+    <t>Outer loop i runs exactly k times (from 0 to k-1). Inner loop j scans the unsorted subarray from 0 to len(A)-1-i, bubbling the maximum remaining element to the right-side wall. Target value is found at A[len(A) - k].</t>
+  </si>
+  <si>
+    <t>O(n) best (when k=1) / O(n · k) average / O(n · k) worst</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary (In-place index swaps)</t>
+  </si>
+  <si>
+    <t>Kth Largest via QuickSelect</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer (Decrease by a Constant Factor / Randomized Pivot Partitioning)</t>
+  </si>
+  <si>
+    <t>The Target Binary Split: Choose a pivot element and partition the array (using Lomuto or Hoare). Check the pivot's resulting index. If it hits the Kth slot, stop. If not, throw away the irrelevant half entirely and recurse only into the surviving side.</t>
+  </si>
+  <si>
+    <t>Run partition helper to find pivot_index. If pivot_index == len(A) - k, return A[pivot_index]. If pivot_index &lt; len(A) - k, recurse right: QuickSelect(pivot_index + 1, end). Else, recurse left: QuickSelect(start, pivot_index - 1).</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary iterative / O(log n) average recursive call stack depth</t>
+  </si>
+  <si>
+    <t>O(n) best if K is the pivot in first iternation/ O(n) average occurs when pivot falls in 95% of the pivot region and reduces atleast 5% in every iteration / O(n²) worst (Worst case occurs if elements are sorted and you consistently select poor, asymmetrical boundary pivots)</t>
+  </si>
+  <si>
+    <t>Kth Largest via Bounded Min-Heap Streaming</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer (Data Structure Shift / Bounded Streaming Buffer)</t>
+  </si>
+  <si>
+    <t>The VIP Club Guard: Build a VIP line with exactly k slots ordered small-to-large (Min-Heap). The weakest link sits at the root door. If a newcomer is stronger than the door guardian, kick the guardian out, push the newcomer in, and re-sort the line.</t>
+  </si>
+  <si>
+    <t>1. Push the first k elements of array A into a Min-Heap. 2. Iterate remaining items from index k to len(A)-1. If item &gt; heap[0], execute heapq.heappushpop(heap, item) to drop the min and maintain size k. 3. Return heap[0] as the final answer.</t>
+  </si>
+  <si>
+    <t>O(n log k) best / O(n log k) average / O(n log k) worst (Provides O(1) instant rejection for elements smaller than the root)</t>
+  </si>
+  <si>
+    <t>O(k) auxiliary space (Strictly bounded footprint; preserves original input array completely)</t>
+  </si>
+  <si>
+    <t>Find Median from Data Stream (Two-Heaps)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Dual Priority Queue Balancing</t>
+  </si>
+  <si>
+    <t>The Balanced Seesaw: Split the incoming data stream into a lower-half group (Max-Heap) and an upper-half group (Min-Heap). Keep the seesaw perfectly level. The median is either the average of the two heavy center points or the peak of the heavier side.</t>
+  </si>
+  <si>
+    <t>1. Add element: If empty or num &lt;= median, push to max_heap (inverted sign); else push to min_heap. 2. Balance: If len(max_heap) &gt; len(min_heap) + 1, pop max_heap and push to min_heap. If len(min_heap) &gt; len(max_heap) + 1, pop min_heap and push to max_heap. 3. Median: If lengths equal, return (max_heap[0] + min_heap[0]) / 2. Else, return root of the larger heap.</t>
+  </si>
+  <si>
+    <t>O(log n) to insert/rebalance / O(1) to find median</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space (to hold all streamed elements across both heap structures)</t>
+  </si>
+  <si>
+    <t>Median via Full Sorting (Brute Force)</t>
+  </si>
+  <si>
+    <t>The Complete Lineup: Line up every single element in the array from smallest to largest using a standard sorting engine, then walk straight to the absolute middle slot to read the value.</t>
+  </si>
+  <si>
+    <t>Sort the entire fixed array A in-place or via copy using a standard O(n log n) library function. Calculate mid = len(A) // 2. If len(A) % 2 != 0, return A[mid]. Else, return (A[mid - 1] + A[mid]) / 2.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst</t>
+  </si>
+  <si>
+    <t>O(1) to O(n) auxiliary (Dependent entirely on the internal implementation of the language's sorting algorithm)</t>
+  </si>
+  <si>
+    <t>Median of Fixed Array via QuickSelect (Optimal)</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / Randomized Pivot Pruning</t>
+  </si>
+  <si>
+    <t>The Blind Bisector: Pick a random element as a pivot. Partition the array into items smaller and larger than the pivot. Check the pivot's index. If it lands exactly on the middle index, stop. If not, throw away the irrelevant side and recurse only into the half containing the middle slot.</t>
+  </si>
+  <si>
+    <t>Target index target = len(A) // 2. Run partition helper returning pivot_idx. If pivot_idx == target, return A[pivot_idx]. If pivot_idx &lt; target, recurse right: QuickSelect(pivot_idx + 1, end, target). Else, recurse left: QuickSelect(start, pivot_idx - 1, target). (Handle even lengths by finding target - 1andtarget).</t>
+  </si>
+  <si>
+    <t>O(n) best / O(n) average / O(n²) worst (Worst case occurs only if poor, unbalanced edge pivots are chosen repeatedly)</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary iterative / O(log n) average recursive stack depth</t>
+  </si>
+  <si>
+    <t>Median via Max-Heap Construction</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer (Structural Heap Optimization)</t>
+  </si>
+  <si>
+    <t>The Pyramid Drain: Convert the entire fixed array into a rigid organizational pyramid (Max-Heap) all at once. Repeatedly chop off the top boss and re-heapify exactly N // 2 times until the median element surfaces at the peak.</t>
+  </si>
+  <si>
+    <t>1. Call bottom-up heapify over the entire fixed array from len(A)//2 - 1 down to 0 to establish a Max-Heap in O(n) time. 2. Run an extraction loop exactly (len(A) // 2) times, swapping the root to the shrinking boundary and sifting down. The root at the final step is your median.</t>
+  </si>
+  <si>
+    <t>O(n) best / O(n log n) average / O(n log n) worst (Build heap phase takes O(n), followed by N//2 extractions which each cost O(log n))</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary space (If array mutation is allowed; completely avoids the two-heap streaming memory allocation footprint)</t>
+  </si>
+  <si>
+    <t>Meeting Rooms I (Can Attend All)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Adjacent Interval Conflict Scan</t>
+  </si>
+  <si>
+    <t>The Schedule Overlay: Sort your calendar appointments chronologically. Walk down the list day-by-day and check if your current meeting wraps up after the very next meeting is scheduled to begin.</t>
+  </si>
+  <si>
+    <t>1. Sort intervals by start time: intervals.sort(). 2. Loop i from 0 to len(intervals) - 1. If i == len(intervals) - 1, next_start = inf; else next_start = intervals[i+1][0]. 3. Boundary check: if intervals[i][1] &gt; next_start, return False. 4. Return True if loop finishes.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst (Dominated by sorting; linear O(n) checking scan)</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary space if sorted in-place</t>
+  </si>
+  <si>
+    <t>Meeting Rooms II (Min Rooms Required)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Chronological Min-Heap Simulation</t>
+  </si>
+  <si>
+    <t>The Active Room Tracker: Sort meetings by start time. As each meeting begins, assign it a room by dropping its end time into a min-heap. Clear out any rooms whose meetings have finished before the next time block starts, and track the peak room count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    1. intervals.sort(). 2. Loop i in range(len(intervals)). Push current end time: heapq.heappush(pq, intervals[i][1]). 3. Track concurrency peak: global_max = max(global_max, len(pq)). 4. Clean up expired rooms: while pq and pq[0] &lt;= next_start_time: heapq.heappop(pq). 5. Return global_max.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst (Sorting costs O(n log n); each element is pushed/popped from heap at most once costing O(n log n))</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space to store concurrent meeting end times in the heap buffer</t>
+  </si>
+  <si>
+    <t>Car Pooling (Look-Ahead Look-up Variant)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Next-Frame Chronological Simulation</t>
+  </si>
+  <si>
+    <t>The Station Radio: Look at the passenger log. Before finishing your current segment, look ahead at the radio dispatch to find the next station's pickup time (next_start_time). Drop off anyone whose destination has already passed before starting the next frame.</t>
+  </si>
+  <si>
+    <t>1. Sort trips by start location. 2. Set next_start_time = trips[i+1][0] (or inf if last). 3. Add passengers and check if current_passengers &gt; capacity. 4. Push (end, passengers) to min-heap. 5. Clear heap using while pq and pq[0][0] &lt;= next_start_time to offload passengers before next pass.</t>
+  </si>
+  <si>
+    <t>Insert Interval (Three-Phase Sequential Sweep)</t>
+  </si>
+  <si>
+    <t>Greedy / Chronological Progress Pointer / State Isolation</t>
+  </si>
+  <si>
+    <t>Initialize i = 0, result = []. 1. Left Phase: while i &lt; n and intervals[i][1] &lt; newInterval[0], append intervals[i], i++. 2. Merge Phase: while i &lt; n and intervals[i][0] &lt;= newInterval[1], merge bounds via min/max into newInterval, i++. Append final newInterval. 3. Right Phase: while i &lt; n, append intervals[i], i++. Auto-handles empty/extreme ranges.</t>
+  </si>
+  <si>
+    <t>The Conveyor Belt: Walk a progress pointer linearly through a conveyor belt of intervals. Left phase drops safe items off into results. Overlap phase rolls colliding items together into a single merged snowball. Right phase collects the snowball and safely packs away all remaining trailing items. (Hint: Draw couple of examples and it becomes clear why merge compares intervals[i][0]&lt;new_interval[1].</t>
+  </si>
+  <si>
+    <t>O(n) best / O(n) average / O(n) worst (Guaranteed single-pass, sequential linear sweep over the list indices)</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space (To build and return the clean, non-overlapping merged results list)</t>
+  </si>
+  <si>
+    <t>Insert Interval (Bail-Index / Dynamic Anchor Variant)</t>
+  </si>
+  <si>
+    <t>Greedy / Index Segmentation / Anchor Overlap Tracking</t>
+  </si>
+  <si>
+    <t>The Clipboard Hand-off: Walk down the list and pack away all early elements. Pause at the exact cutoff index (bail_index), drop your new interval onto the clipboard, and then resume scanning the remainder of the line, dynamically stretching your clipboard's trailing frame whenever a collision occurs.</t>
+  </si>
+  <si>
+    <t>1. Loop i from 0 to N-1: if intervals[i][1] &lt; new_interval[0], append to result and increment bail_index. Else, break. 2. Append new_interval directly to result. 3. Loop i from bail_index to N-1: if result[-1][1] &lt; intervals[i][0], append intervals[i]. Else, mutate result[-1] via in-place min/max bound calculations.</t>
+  </si>
+  <si>
+    <t>O(n) best / O(n) average / O(n) worst (Processes the elements via two clean, separate sequential linear passes)</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space (To build and isolate the fresh, non-overlapping array blocks)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -665,6 +1073,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -674,7 +1089,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -697,15 +1112,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -715,6 +1164,20 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1020,16 +1483,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="28.6640625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="48.1640625" style="3" customWidth="1"/>
     <col min="2" max="2" width="41.33203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="56.5" style="4" customWidth="1"/>
-    <col min="4" max="4" width="58.1640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="56.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="58.1640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="41.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="28.6640625" style="3"/>
+    <col min="6" max="6" width="35.83203125" style="3" customWidth="1"/>
+    <col min="7" max="16384" width="28.6640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22" x14ac:dyDescent="0.25">
@@ -1039,56 +1502,56 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="69" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="92" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1099,16 +1562,16 @@
       <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1116,19 +1579,19 @@
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1136,19 +1599,19 @@
       <c r="A6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1156,19 +1619,19 @@
       <c r="A7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1176,19 +1639,19 @@
       <c r="A8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>39</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1196,19 +1659,19 @@
       <c r="A9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>43</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1216,19 +1679,19 @@
       <c r="A10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1236,19 +1699,19 @@
       <c r="A11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1259,16 +1722,16 @@
       <c r="B12" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1276,19 +1739,19 @@
       <c r="A13" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1296,23 +1759,516 @@
       <c r="A14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>73</v>
       </c>
     </row>
+    <row r="15" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="176" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="198" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="198" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90D5E7E3-4B6F-0647-827B-D0D81B8D09D9}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="41" customWidth="1"/>
+    <col min="3" max="3" width="33.1640625" customWidth="1"/>
+    <col min="4" max="4" width="38.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.33203125" customWidth="1"/>
+    <col min="6" max="6" width="28.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" spans="1:8" ht="45" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="176" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="132" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="154" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="242" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="198" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="198" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added Bit wise algorithms
</commit_message>
<xml_diff>
--- a/DSA/Sorting/dsa_cheatsheet.xlsx
+++ b/DSA/Sorting/dsa_cheatsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/balaji.gurusala/Documents/Code/coding/DSA/Sorting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE417D1-D94F-EB43-B21C-E9B0F367709A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9BEB72-7ECC-1144-9EB5-949EEB1B5A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38580" yWindow="600" windowWidth="34560" windowHeight="20600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Algorithms" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="258">
   <si>
     <t>Algorithm / Concept</t>
   </si>
@@ -1013,6 +1013,168 @@
   </si>
   <si>
     <t>O(n) auxiliary space (To build and isolate the fresh, non-overlapping array blocks)</t>
+  </si>
+  <si>
+    <t>Employee Free Time (Flatten &amp; Sort Variant)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Interval Inversion</t>
+  </si>
+  <si>
+    <t>The Master Calendar: Dump every single person's calendar items into one big messy pile. Sort the entire pile chronologically, zip all overlapping busy blocks together into thick blocks, and collect the quiet gaps left between those blocks.</t>
+  </si>
+  <si>
+    <t>1. Flatten schedule into all_intervals. 2. Sort via key=lambda x: x[0]. 3. Standard Merge Interval loop to build merged_intervals. 4. Collect gaps: loop i from 0 to len(merged_intervals)-2, appending [merged_intervals[i][1], merged_intervals[i+1][0]].</t>
+  </si>
+  <si>
+    <t>O(N log N) best / O(N log N) average / O(N log N) worst (Where N is the total number of individual interval blocks)</t>
+  </si>
+  <si>
+    <t>O(N) auxiliary space to house the flattened copy of the array dataset</t>
+  </si>
+  <si>
+    <t>Employee Free Time (Full-Heap Population Variant)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Out-of-Place Heapification</t>
+  </si>
+  <si>
+    <t>The Megaphone Collection: Read every single employee's schedule and throw every interval block into one big massive bucket-heap all at once. Repeatedly pull the earliest chronologically scheduled block off the top of the pile to build a linear timeline, zipping overrides together and grabbing the quiet spaces between them.</t>
+  </si>
+  <si>
+    <t>1. Double nested loops push every interval into min_heap tracking (start, end). 2. Initialize merged_intervals with float('-inf') bounds. 3. While heap exists: pop (start, end). If start &gt; merged_intervals[-1][1], append [start, end]. Else, update merged_intervals[-1][1] = max(merged_intervals[-1][1], end). 4. Collect intervals via linear gap slice loop.</t>
+  </si>
+  <si>
+    <t>O(N log N) best / O(N log N) average / O(N log N) worst (Where N is the total number of intervals across all profiles; every item triggers a heap push/pop transition)</t>
+  </si>
+  <si>
+    <t>O(N) auxiliary space (The priority queue expands dynamically to hold the entire collection of timeline elements simultaneously)</t>
+  </si>
+  <si>
+    <t>Employee Free Time (K-Way Heap Merge Variant)</t>
+  </si>
+  <si>
+    <t>Space-Time Trade-off / Bounded Priority Queue Fusion / K-Way Selection</t>
+  </si>
+  <si>
+    <t>The Concurrency Card Dealer: Every employee holds an independent pre-sorted stack of appointment cards. Place only the top card from each stack onto a tiny table-heap. Pop the absolute earliest card, merge its limits into your master results layout, and instantly replace it with the next sequential card from that specific employee's hand.</t>
+  </si>
+  <si>
+    <t>1. Initialize heap with the 0th interval of each employee chunk via (item[0], item[1], item, 0). 2. Merged_intervals begins with float('-inf') bounds. 3. While heap exists: pop element, merge into result[-1] via max bounds or append. 4. If pos + 1 &lt; len(employee), push (pos+1) element back onto the min-heap. 5. Interleave linear gap collection pass.</t>
+  </si>
+  <si>
+    <t>O(N log K) best / O(N log K) average / O(N log K) worst (Where N is the total number of intervals globally, and K is the number of individual employee tracks; drastically outperforms O(N log N) when K is small)</t>
+  </si>
+  <si>
+    <t>O(K) auxiliary space (The priority queue structure size footprint is strictly capped to store at most K tracking nodes at any single instant)</t>
+  </si>
+  <si>
+    <t>Interval Intersection (Merge &amp; Sort)</t>
+  </si>
+  <si>
+    <t>Brute Force / Exhaustive Flattening</t>
+  </si>
+  <si>
+    <t>The Blended Deck: Dump both lists together into one big pile, sort them chronologically by their start coordinates, and then do a linear forward scan to see if adjacent blocks crash together.</t>
+  </si>
+  <si>
+    <t>1. Interleave firstList and secondList elements into merged_intervals. 2. Sort via key=lambda x: x. 3. Loop i from 0 to len(merged_intervals)-2. If current.end &gt;= next.start, append [max(starts), min(ends)] intersection to result.</t>
+  </si>
+  <si>
+    <t>O((N+M) log(N+M)) best/avg/worst (Where N and M are the sizes of the two lists; completely dominated by the explicit sorting pass)</t>
+  </si>
+  <si>
+    <t>O(N + M) auxiliary space to house the combined and flattened array copy</t>
+  </si>
+  <si>
+    <t>Interval Intersection (Synchronized Two-Pointer Sweep)</t>
+  </si>
+  <si>
+    <t>The Parallel Conveyor Belts: Put a tracking hand on both sorted lists simultaneously. If the current two intervals touch, record their overlapping segment using max(starts) and min(ends). Then, pick up the hand resting on the interval that finishes earlier and slide it forward.</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Two-Pointer Coordinate March</t>
+  </si>
+  <si>
+    <t>While i &lt; len(list1) and j &lt; len(list2): 1. Check overlap: if list1[i].end &gt;= list2[j].start and list2[j].end &gt;= list1[i].start, append [max(starts), min(ends)]. 2. Advance: if list1[i].end &lt;= list2[j].end, i++; else, j++. Auto-handles distinct or nested overlaps.</t>
+  </si>
+  <si>
+    <t>O(N + M) best/avg/worst (Guaranteed single-pass linear sweep; each element is visited at most once)</t>
+  </si>
+  <si>
+    <t>O(1) constant auxiliary space (Operates completely in-place on the pre-sorted input lists)</t>
+  </si>
+  <si>
+    <t>3Sum Smaller (Count Triplets)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Anchor-and-Pincer Multi-Pointer Sweep</t>
+  </si>
+  <si>
+    <t>The Fixed Pivot Anchor: Pin down an anchor element on the left side of a sorted line. Drop a traditional two-pointer pincer scan ahead of it. If the ends crash below the target, sweep all intermediate elements at once using index math, slide the left hand forward, and repeat.</t>
+  </si>
+  <si>
+    <t>1. Sort array. 2. Outer loop i from 0 to N-3 acts as the fixed anchor. 3. Inner pincer while left &lt; right (starting at i+1): if sum &gt;= new_target, decrement right. Else, accumulate count += (right - left) and increment left. 4. Return total global count.</t>
+  </si>
+  <si>
+    <t>O(n²) best / O(n²) average / O(n²) worst (Pre-sorting takes O(n log n); outer loop runs N times nesting a linear O(n) two-pointer scan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> O(1) constant auxiliary space (Operates entirely in-place via pointer indexes)</t>
+  </si>
+  <si>
+    <t>Top K Frequent Words (Bounded Min-Heap)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Custom Comparator Bounded Streaming</t>
+  </si>
+  <si>
+    <t>The Smart VIP Line: Build an elite line capped at size K. Parents are smaller than children on frequencies, but alphabetically larger on equal scores. Pop automatically removes weak scores and bad names, ensuring the best candidates survive.</t>
+  </si>
+  <si>
+    <t>1. Counter(words) maps frequency. 2. Loop entries pushing custom objects to a min-heap. Object uses custom __lt__ comparing frequency directly but string inversely via word &gt; other.word. 3. If len(heap) &gt; k, execute heappop(). 4. Collect and reverse output.</t>
+  </si>
+  <si>
+    <t>O(N log K) best / O(N log K) average / O(N log K) worst (Where N is the count of unique words. Significantly faster than full sorting when K is small)</t>
+  </si>
+  <si>
+    <t>O(N) auxiliary space (To maintain the hash table counter and the active priority queue footprint)</t>
+  </si>
+  <si>
+    <t>QuickSelect with Custom Sorting Suffix</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / QuickSelect Linear Rank Reduction</t>
+  </si>
+  <si>
+    <t>The Target Split: Group the elements into a unique keys list. Run an randomized pivot selection loop to isolate the K highest elements to the left chunk of the list in linear time, then sort only that tiny extracted partition.</t>
+  </si>
+  <si>
+    <t>1. Unique words list built from hash map counts. 2. Run recursive QuickSelect with Lomuto partitioning to isolate the top K ranks around a random pivot. 3. Sift conditions: if count &gt; pivot or (count == pivot and word &lt; pivot_word), slide left boundary. 4. Slice words[:k] and execute sorted(key=lambda x: (-count[x], x)).</t>
+  </si>
+  <si>
+    <t>O(N + K log K) best / O(N + K log K) average / O(N² + K log K) worst (Average time is dominated by linear O(N) QuickSelect followed by a fast K log K sort of the isolated target slice)</t>
+  </si>
+  <si>
+    <t>O(N) auxiliary space (To manage unique word collections and hash tables)</t>
+  </si>
+  <si>
+    <t>3Sum (Unique Triplets Tracking)</t>
+  </si>
+  <si>
+    <t>Transform &amp; Conquer / Pre-Sorting / Anchor-with-Two-Pointer-Pincer</t>
+  </si>
+  <si>
+    <t>The Static Anchor &amp; Moving Pincer: Sort the array to group duplicates together. Lock down an anchor pointer on the left. If the anchor is positive, abort early. Otherwise, launch a two-pointer pincer sweep ahead, snapping inward on matches while skidding past duplicate elements.</t>
+  </si>
+  <si>
+    <t>1. arr.sort(). 2. Outer loop i from 0 to N-1: if arr[i] &gt; 0 break; if i &gt; 0 and arr[i] == arr[i-1] continue. 3. Call twoSum helper with left = i+1, right = N-1, target = -arr[i]. 4. Inside twoSum: while left &lt; right, match gives left++, right--, then run while left &lt; right and arr[left] == arr[left-1] left++ to drop duplicates.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n²) average / O(n²) worst (Pruning allows best case to exit early on positive arrays; dominated by quadratic loops)</t>
+  </si>
+  <si>
+    <t>O(1) constant auxiliary space (Operates completely in-place on the pre-sorted input array structures)</t>
   </si>
 </sst>
 </file>
@@ -1153,7 +1315,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1165,9 +1327,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1176,8 +1335,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1483,7 +1642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="28.6640625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.1640625" style="3" customWidth="1"/>
@@ -1775,324 +1934,504 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="154" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="88" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="17" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="132" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>85</v>
       </c>
       <c r="F17" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="88" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="19" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="110" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="20" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="132" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="22" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B22" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="176" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="23" spans="1:6" ht="176" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="198" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="24" spans="1:6" ht="198" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="110" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="25" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="154" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="26" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="132" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="132" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B28" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>181</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="154" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="154" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B30" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C30" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="198" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+    <row r="31" spans="1:6" ht="198" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B31" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="154" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="32" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B32" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C32" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>203</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="176" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="176" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -2114,34 +2453,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="45" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2218,10 +2557,10 @@
       <c r="D6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="3" t="s">
         <v>126</v>
       </c>
     </row>
@@ -2238,10 +2577,10 @@
       <c r="D7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="3" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2258,10 +2597,10 @@
       <c r="D8" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>128</v>
       </c>
     </row>

</xml_diff>